<commit_message>
feat(services): directly submit new services to manager approval with push notifications
</commit_message>
<xml_diff>
--- a/web/Cariler.xlsx
+++ b/web/Cariler.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A371"/>
+  <dimension ref="A1:A374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="112" customWidth="1" min="1" max="1"/>
@@ -717,2337 +717,2358 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BABUNEC ERZURUM KAHVALTI DÜNYASI  YASEMİN DEMİREL</t>
+          <t>AZİZCAN ISIYEL</t>
         </is>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>BAHEM PERAKENDE GIDA HAYV.İNŞ.TARIM İTH.İHR.SAN.VE TİC.LTD.ŞTİ.</t>
+          <t>BABUNEC ERZURUM KAHVALTI DÜNYASI  YASEMİN DEMİREL</t>
         </is>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>BAK İMALAT</t>
+          <t>BAHEM PERAKENDE GIDA HAYV.İNŞ.TARIM İTH.İHR.SAN.VE TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BALCI İFRAN-MUHAMMED İRFAN ŞANLI</t>
+          <t>BAK İMALAT</t>
         </is>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BANKA ENPARA ŞAHSİ</t>
+          <t>BALCI İFRAN-MUHAMMED İRFAN ŞANLI</t>
         </is>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BANKA ENPARA ŞİRKET</t>
+          <t>BANKA ENPARA ŞAHSİ</t>
         </is>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BANKA YAPI KREDİ</t>
+          <t>BANKA ENPARA ŞİRKET</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BARIŞ AKADEMİ - BARIŞ VAROL İNSUYU</t>
+          <t>BANKA YAPI KREDİ</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BAŞKAYA SAKATAT ET VE ET ÜRÜNLERİ</t>
+          <t>BARIŞ AKADEMİ - BARIŞ VAROL İNSUYU</t>
         </is>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BAYPA MOBİLYA - AYHAN DEMİR</t>
+          <t>BAŞKAYA SAKATAT ET VE ET ÜRÜNLERİ</t>
         </is>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BEKEN AYAKKABI MUHAMMED</t>
+          <t>BAYPA MOBİLYA - AYHAN DEMİR</t>
         </is>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BEKİR TEK</t>
+          <t>BEKEN AYAKKABI MUHAMMED</t>
         </is>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BERF İLAÇ VE KOZMETİK SAN.TİC.LTD.ŞTİ.</t>
+          <t>BEKİR TEK</t>
         </is>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BEŞYILDIZ PETROL ÜRÜNLERİ TAŞ. GIDA İNŞ. MLZ. TRZ. SAN. VE TİC . AŞ.</t>
+          <t>BERF İLAÇ VE KOZMETİK SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Bİ DUNYA DETAY ZÜCCACİYE LTD.ŞTİ</t>
+          <t>BEŞYILDIZ PETROL ÜRÜNLERİ TAŞ. GIDA İNŞ. MLZ. TRZ. SAN. VE TİC . AŞ.</t>
         </is>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>Bilişimpos Otomasyon Yazılım Sanayi Ve Ticaret Limited Şirketi</t>
+          <t>Bİ DUNYA DETAY ZÜCCACİYE LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>BİREN  ENERJİ ELEKTRİK MALZ.İNŞ.TURİZM GIDA SAN. VE TİC. LTD.ŞTİ.</t>
+          <t>Bilişimpos Otomasyon Yazılım Sanayi Ve Ticaret Limited Şirketi</t>
         </is>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>BİRENSES ENERJİ ELEKTRİK ELEKTRONİK İNŞAAT MALZEMELERİ İNŞAAT TAAHHÜT SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>BİREN  ENERJİ ELEKTRİK MALZ.İNŞ.TURİZM GIDA SAN. VE TİC. LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>BNG LOJİSTİK</t>
+          <t>BİRENSES ENERJİ ELEKTRİK ELEKTRONİK İNŞAAT MALZEMELERİ İNŞAAT TAAHHÜT SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>BOL BOL TAVUK DÖNER</t>
+          <t>BNG LOJİSTİK</t>
         </is>
       </c>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>BOLİVİA ZÜCCACİYE</t>
+          <t>BOL BOL TAVUK DÖNER</t>
         </is>
       </c>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>BÖRÜ KİTAP KIRTASİYE - HABİP ÇOLAK</t>
+          <t>BOLİVİA ZÜCCACİYE</t>
         </is>
       </c>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>BUHARA SAĞLIK HİZMETLERİ A.Ş.</t>
+          <t>BÖRÜ KİTAP KIRTASİYE - HABİP ÇOLAK</t>
         </is>
       </c>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Büşra Akpunar - Moda Aksesuar</t>
+          <t>BUHARA SAĞLIK HİZMETLERİ A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>CAFE BEY -AHMET YILMAZ</t>
+          <t>BURAK AĞCAKAYA</t>
         </is>
       </c>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>CAFE DE CINEMA FİLM SİNEMA REK.YİY.HİZ. VE KAŞE İML.LTD.ŞTİ</t>
+          <t>Büşra Akpunar - Moda Aksesuar</t>
         </is>
       </c>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>CAHİT DAL</t>
+          <t>CAFE BEY -AHMET YILMAZ</t>
         </is>
       </c>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>CESO TEKSTIL - CASIM POLAT</t>
+          <t>CAFE DE CINEMA FİLM SİNEMA REK.YİY.HİZ. VE KAŞE İML.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>CHEFF TANTUNI</t>
+          <t>CAHİT DAL</t>
         </is>
       </c>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>CHOCOLADE BOUTİQUE ALANYA - ÖZLEM GÖKTEPE</t>
+          <t>CESO TEKSTIL - CASIM POLAT</t>
         </is>
       </c>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>CHOCOLADE ELAZIĞ - FERHAT YILDIRIM</t>
+          <t>CHEFF TANTUNI</t>
         </is>
       </c>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>CİMİLLİ EV TEKSTİL TİC.SAN.LTD. ŞTİ.</t>
+          <t>CHOCOLADE BOUTİQUE ALANYA - ÖZLEM GÖKTEPE</t>
         </is>
       </c>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ÇAĞRI KİTAP KIRTASİYE DAĞ.LTD.ŞTİ.</t>
+          <t>CHOCOLADE ELAZIĞ - FERHAT YILDIRIM</t>
         </is>
       </c>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ÇINARLI KİTAP CAFE</t>
+          <t>CİMİLLİ EV TEKSTİL TİC.SAN.LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ÇİFTÇİLER MANAV - SERPİL ÇİFTÇİ</t>
+          <t>ÇAĞRI KİTAP KIRTASİYE DAĞ.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ÇİFTÇİLER TARIM TARIMSAL SULAMA VE GÜNEŞ ENERJİSİ SÎSTEMLERİ</t>
+          <t>ÇINARLI KİTAP CAFE</t>
         </is>
       </c>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ÇİFTSAN TURİZM EMLAK İNŞAAT YAPI SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>ÇİFTÇİLER MANAV - SERPİL ÇİFTÇİ</t>
         </is>
       </c>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ÇİZGİ TELEKOMÜNİKASYON ANONİM ŞİRKETİ ÇİZGİ</t>
+          <t>ÇİFTÇİLER TARIM TARIMSAL SULAMA VE GÜNEŞ ENERJİSİ SÎSTEMLERİ</t>
         </is>
       </c>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ÇİZMELİOĞLU SÜT  LTD.ŞTİ.</t>
+          <t>ÇİFTSAN TURİZM EMLAK İNŞAAT YAPI SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>DEĞİRMEN RESTORANT</t>
+          <t>ÇİZGİ TELEKOMÜNİKASYON ANONİM ŞİRKETİ ÇİZGİ</t>
         </is>
       </c>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>DEVRİ ALEM GIDA ŞARKÜTERİ VE KAHVALTI İŞL.SAN.TİC.LTD.ŞTİ.</t>
+          <t>ÇİZMELİOĞLU SÜT  LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>D-MARKET ELEKTRONİK HİZMETLER VE TİCARET ANONİM ŞİRKETİ</t>
+          <t>DEĞİRMEN RESTORANT</t>
         </is>
       </c>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>DOĞAN KIRTASİYE - YILMAZ DOĞAN</t>
+          <t>DEVRİ ALEM GIDA ŞARKÜTERİ VE KAHVALTI İŞL.SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>DOĞU ELEKTROMARKET - ZAFER KAZA</t>
+          <t>D-MARKET ELEKTRONİK HİZMETLER VE TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>DÖNERCİ HACIBABANIN YERİ LOKANTASI  LTD. ŞTİ</t>
+          <t>DOĞAN KIRTASİYE - YILMAZ DOĞAN</t>
         </is>
       </c>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>DÖNMEZ ET ÜRÜNLERİ - MUHARREM DÖNMEZ</t>
+          <t>DOĞU ELEKTROMARKET - ZAFER KAZA</t>
         </is>
       </c>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>DURAKOĞULLARI GIDA HAYVANCILIK TURİZM SEYAHAT VE İNŞAAT TAAHHÜT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
+          <t>DÖNERCİ HACIBABANIN YERİ LOKANTASI  LTD. ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Efdal Kuru Gıda - Memet Bilici</t>
+          <t>DÖNMEZ ET ÜRÜNLERİ - MUHARREM DÖNMEZ</t>
         </is>
       </c>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>EGEMEN ASLAN ATILIM MARKET</t>
+          <t>DURAKOĞULLARI GIDA HAYVANCILIK TURİZM SEYAHAT VE İNŞAAT TAAHHÜT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>EKONOMİK ALIŞVERİŞ MERKEZİ MARKETÇİLİK TİC. SAN. LTD. ŞTİ</t>
+          <t>Efdal Kuru Gıda - Memet Bilici</t>
         </is>
       </c>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ELİF MARKET - CENNET PEHLİVAN</t>
+          <t>EGEMEN ASLAN ATILIM MARKET</t>
         </is>
       </c>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>ELİSYA ÇİKOLATA KAFE SAN. VE TİC. LTD.ŞTİ.</t>
+          <t>EKONOMİK ALIŞVERİŞ MERKEZİ MARKETÇİLİK TİC. SAN. LTD. ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>ELİT MATBAA - İSRAFİL TOPARLAK</t>
+          <t>ELİF MARKET - CENNET PEHLİVAN</t>
         </is>
       </c>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>EnPOS Bilişim Sanayi ve Ticaret A.Ş.</t>
+          <t>ELİSYA ÇİKOLATA KAFE SAN. VE TİC. LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>ERATA EĞİTİM SAĞLIK DAN.HİZ.İNŞ.TAAH.GIDA SAN.VE TİC. AŞ.</t>
+          <t>ELİT MATBAA - İSRAFİL TOPARLAK</t>
         </is>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ERAY TEKNOLOJİ SANAYİ VE TİCARET A.Ş.</t>
+          <t>EnPOS Bilişim Sanayi ve Ticaret A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>ERCAN AKDAĞ</t>
+          <t>ERATA EĞİTİM SAĞLIK DAN.HİZ.İNŞ.TAAH.GIDA SAN.VE TİC. AŞ.</t>
         </is>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>EREN GIDA - ONUR EREN</t>
+          <t>ERAY TEKNOLOJİ SANAYİ VE TİCARET A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>ERENLER MANAVI - MENSUR BİLMEZ</t>
+          <t>ERCAN AKDAĞ</t>
         </is>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>ERGİN GÜLER</t>
+          <t>EREN GIDA - ONUR EREN</t>
         </is>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>ER-KALE İNŞ.TAAH.MOB.SAN.TİC.LTD.ŞTİ.</t>
+          <t>ERENLER MANAVI - MENSUR BİLMEZ</t>
         </is>
       </c>
     </row>
     <row r="99" ht="20" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>ERKAN ÇAKMAK</t>
+          <t>ERGİN GÜLER</t>
         </is>
       </c>
     </row>
     <row r="100" ht="20" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>ERKAR İŞ SAĞLIĞI VE GÜVENLİĞİ EĞT. DAN. TURZ.SAN. VE TİC. LTD.ŞTİ</t>
+          <t>ER-KALE İNŞ.TAAH.MOB.SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="101" ht="20" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>ERKENT SİTESİ</t>
+          <t>ERKAN ÇAKMAK</t>
         </is>
       </c>
     </row>
     <row r="102" ht="20" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Erko Plastik Ambalaj Gıda San.Tic.Ltd.Şti.</t>
+          <t>ERKAR İŞ SAĞLIĞI VE GÜVENLİĞİ EĞT. DAN. TURZ.SAN. VE TİC. LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>ER-ONUR İNŞAAT EMLAK OTOMOTİV - NECMETTİN TOPŞAKLI</t>
+          <t>ERKENT SİTESİ</t>
         </is>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>ERTUĞRA İNŞ.TAAHD.GAZ.ELEKT.ELEKTRONİK GIDA SAN.LTD.ŞTİ.</t>
+          <t>Erko Plastik Ambalaj Gıda San.Tic.Ltd.Şti.</t>
         </is>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>ERUZURUM GÜLER ZÜCCACİYE DAY.TÜK.MAD.TİC. SAN.LTD.ŞTİ.</t>
+          <t>ER-ONUR İNŞAAT EMLAK OTOMOTİV - NECMETTİN TOPŞAKLI</t>
         </is>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM AĞIZ VE DİŞ SAĞLIĞI MERKEZİ</t>
+          <t>ERTUĞRA İNŞ.TAAHD.GAZ.ELEKT.ELEKTRONİK GIDA SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM BİLGİSAYAR TİC.LTD.ŞTİ</t>
+          <t>ERUZURUM GÜLER ZÜCCACİYE DAY.TÜK.MAD.TİC. SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM ELEKTRONİK SAN.LTD.ŞTİ</t>
+          <t>ERZURUM AĞIZ VE DİŞ SAĞLIĞI MERKEZİ</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM ENERJİ ÜRETİM DAĞITIM DOĞALGAZ PETROL METAL TAŞ. SAN. VE TİC. A.Ş</t>
+          <t>ERZURUM BİLGİSAYAR TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM EVLERİ - SİYAMİ DEMİR</t>
+          <t>ERZURUM ELEKTRONİK SAN.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM HAYVANCILIK İNŞAAT TAAH.GIDA TURZ. OTOMOTİV SAN. VE TİC. LTD.ŞTİ.</t>
+          <t>ERZURUM ENERJİ ÜRETİM DAĞITIM DOĞALGAZ PETROL METAL TAŞ. SAN. VE TİC. A.Ş</t>
         </is>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM KİTAP MERKEZİ LTD.ŞTİ.</t>
+          <t>ERZURUM EVLERİ - SİYAMİ DEMİR</t>
         </is>
       </c>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM KÜLTÜR EĞİTİM KİTAP KIRTASİYE YAYIN ELEK. İNŞ.TAAH.TİC.LTD.ŞTİ</t>
+          <t>ERZURUM HAYVANCILIK İNŞAAT TAAH.GIDA TURZ. OTOMOTİV SAN. VE TİC. LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="114" ht="20" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM MOTOR OTOMOTİV TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
+          <t>ERZURUM KİTAP MERKEZİ LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="115" ht="20" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM SPOR KÜLTÜR SANAT ETKİNLİĞİ VE İŞLETMECİLİĞİ TİC. SAN. ANONİM. ŞİRKETİ.</t>
+          <t>ERZURUM KÜLTÜR EĞİTİM KİTAP KIRTASİYE YAYIN ELEK. İNŞ.TAAH.TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="116" ht="20" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM TEKNİK ELEKTRONİK SAN.TİC.LTD.ŞTİ.</t>
+          <t>ERZURUM MOTOR OTOMOTİV TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="117" ht="20" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>ERZURUM TİCARET BORSASI TARIM VE HAYVANCILIĞI GELİŞTİRME A.Ş.</t>
+          <t>ERZURUM SPOR KÜLTÜR SANAT ETKİNLİĞİ VE İŞLETMECİLİĞİ TİC. SAN. ANONİM. ŞİRKETİ.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>ES-ER MÜHENDİSLİK İNŞ.TAAH. SAN.TİC.LTD.ŞTİ</t>
+          <t>ERZURUM TEKNİK ELEKTRONİK SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="119" ht="20" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>ESLEM AYDINLATMA ELEKTRİK İNŞ.TAAH.HEDİYELİK EŞYA TİC.VE SAN.LTD.ŞTİ</t>
+          <t>ERZURUM TİCARET BORSASI TARIM VE HAYVANCILIĞI GELİŞTİRME A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="120" ht="20" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>ESTOZA İNŞAAT TAAHHÜT İNŞAAT MALZEMELERİ PEYZAJ TEKNOLOJİ LOKANTACILIK SANAYİ TİCARET LTD.ŞTİ.</t>
+          <t>ES-ER MÜHENDİSLİK İNŞ.TAAH. SAN.TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>ET VE SÜT KURUMU ERZURUM ET KOMBİNASI MÜDÜRLÜĞÜ</t>
+          <t>ESLEM AYDINLATMA ELEKTRİK İNŞ.TAAH.HEDİYELİK EŞYA TİC.VE SAN.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>ETÜ MÜHENDİSLİK KANTNİ</t>
+          <t>ESTOZA İNŞAAT TAAHHÜT İNŞAAT MALZEMELERİ PEYZAJ TEKNOLOJİ LOKANTACILIK SANAYİ TİCARET LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>EVREN SÜT ÜRÜNLERİ</t>
+          <t>ET VE SÜT KURUMU ERZURUM ET KOMBİNASI MÜDÜRLÜĞÜ</t>
         </is>
       </c>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>FATİH KÖMÜRCÜ - SEFA TİCARET</t>
+          <t>ETÜ MÜHENDİSLİK KANTNİ</t>
         </is>
       </c>
     </row>
     <row r="125" ht="20" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>FREDDY MUHAMMED LÜTFİ ÖZDEMİR</t>
+          <t>EVREN SÜT ÜRÜNLERİ</t>
         </is>
       </c>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>FULYA GÜVEN</t>
+          <t>FATİH KÖMÜRCÜ - SEFA TİCARET</t>
         </is>
       </c>
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>FURKAN RESTORANT LTD.ŞTİ.</t>
+          <t>FREDDY MUHAMMED LÜTFİ ÖZDEMİR</t>
         </is>
       </c>
     </row>
     <row r="128" ht="20" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>GECE DÖNERCİSİ EREN USTA - GAMZE TANHAŞ</t>
+          <t>FULYA GÜVEN</t>
         </is>
       </c>
     </row>
     <row r="129" ht="20" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GENCEHAN GIDA TEMİZLİK ÜRÜNLERİ OTOMOTİV SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
+          <t>FURKAN RESTORANT LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="130" ht="20" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>GÖÇ MARKET - BÜLENT ERGİN</t>
+          <t>GECE DÖNERCİSİ EREN USTA - GAMZE TANHAŞ</t>
         </is>
       </c>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GÖKÇE KUYUMCULUK SAN. TARIM ÜRÜN TİC. LTD. ŞTİ.</t>
+          <t>GENCEHAN GIDA TEMİZLİK ÜRÜNLERİ OTOMOTİV SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GÖRSEL ORG.GIDA - ABDULHADİ KÜÇÜK</t>
+          <t>GÖÇ MARKET - BÜLENT ERGİN</t>
         </is>
       </c>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GÜLİSTAN MANAVI</t>
+          <t>GÖKÇE KUYUMCULUK SAN. TARIM ÜRÜN TİC. LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GÜNDOĞDU ASANSOR</t>
+          <t>GÖRSEL ORG.GIDA - ABDULHADİ KÜÇÜK</t>
         </is>
       </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GÜNDOĞDU MEFRUŞAT ÇEZÜCCACİYE HALI TEKSTİTH İHR SAN TİC LTD</t>
+          <t>GÜLİSTAN MANAVI</t>
         </is>
       </c>
     </row>
     <row r="136" ht="20" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GÜNDÜZ MARKET - MURAT GÜNDÜZ</t>
+          <t>GÜNDOĞDU ASANSOR</t>
         </is>
       </c>
     </row>
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>GÜNEŞ KOLEJİ</t>
+          <t>GÜNDOĞDU MEFRUŞAT ÇEZÜCCACİYE HALI TEKSTİTH İHR SAN TİC LTD</t>
         </is>
       </c>
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>GÜNEŞ OTOMASYON-ABDURREHİM GÜNEŞ</t>
+          <t>GÜNDÜZ MARKET - MURAT GÜNDÜZ</t>
         </is>
       </c>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GÜNEYLER AVM - MEHMEY GÜNEY</t>
+          <t>GÜNEŞ KOLEJİ</t>
         </is>
       </c>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>GÜNEYLER LÜKS HIRDAVAT VE GIDA TİC.SAN.LTD.ŞTİ.</t>
+          <t>GÜNEŞ OTOMASYON-ABDURREHİM GÜNEŞ</t>
         </is>
       </c>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GÜNEYLER MAĞAZACILIK TİCARET SAN. LTD. ŞTİ.</t>
+          <t>GÜNEYLER AVM - MEHMEY GÜNEY</t>
         </is>
       </c>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>HACEGAN MERKEZ</t>
+          <t>GÜNEYLER LÜKS HIRDAVAT VE GIDA TİC.SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>HACI BABA LOKANTA GIDA TURİZM LTD.ŞTİ.</t>
+          <t>GÜNEYLER MAĞAZACILIK TİCARET SAN. LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>HAKİMSAN MEKANİK A.Ş.</t>
+          <t>HACEGAN MERKEZ</t>
         </is>
       </c>
     </row>
     <row r="145" ht="20" customHeight="1">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>HAKİMSAN MÜHENDİSLİK LTD.ŞTİ.</t>
+          <t>HACI BABA LOKANTA GIDA TURİZM LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="146" ht="20" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>HAMZA GÜLLÜCE - ÇAY DÜNYASI GÜLLÜCE TİCARET</t>
+          <t>HAKİMSAN MEKANİK A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="147" ht="20" customHeight="1">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>HASAN GÜNDÜZ</t>
+          <t>HAKİMSAN MÜHENDİSLİK LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>HASAN GÜNEŞ</t>
+          <t>HAMZA GÜLLÜCE - ÇAY DÜNYASI GÜLLÜCE TİCARET</t>
         </is>
       </c>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>HASAN İSLAM GÜNEY</t>
+          <t>HASAN GÜNDÜZ</t>
         </is>
       </c>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>HDŞ GRUP BAHARAT GIDA KOZ.BİLG.İLET.TEM.İNŞ.İHT.MAD.PAZ.SAN. VE TİC.LTD.ŞTİ.</t>
+          <t>HASAN GÜNEŞ</t>
         </is>
       </c>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>HEPSİ BURADA</t>
+          <t>HASAN İSLAM GÜNEY</t>
         </is>
       </c>
     </row>
     <row r="152" ht="20" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>HG AYAKKABI - HALİL GÜNAY</t>
+          <t>HDŞ GRUP BAHARAT GIDA KOZ.BİLG.İLET.TEM.İNŞ.İHT.MAD.PAZ.SAN. VE TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>HİLAL TÜRKYILMAZ</t>
+          <t>HEPSİ BURADA</t>
         </is>
       </c>
     </row>
     <row r="154" ht="20" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>HUZURUM SAMSUN</t>
+          <t>HG AYAKKABI - HALİL GÜNAY</t>
         </is>
       </c>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>HÜNKAR RESTORAN</t>
+          <t>HİLAL TÜRKYILMAZ</t>
         </is>
       </c>
     </row>
     <row r="156" ht="20" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>IDEASOFT YAZILIM SAN. VE TİC. A.Ş.</t>
+          <t>HUZURUM SAMSUN</t>
         </is>
       </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>İBRAHİM AYYILMAZ - AYYILMAZ</t>
+          <t>HÜNKAR RESTORAN</t>
         </is>
       </c>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>İBRAHİM DEMİR - KOTAN MARKET</t>
+          <t>IDEASOFT YAZILIM SAN. VE TİC. A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>İKBAL TAVUK DÖNER -  KADİR YAVUZ</t>
+          <t>İBRAHİM AYYILMAZ - AYYILMAZ</t>
         </is>
       </c>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>İLYAS TOSUN</t>
+          <t>İBRAHİM DEMİR - KOTAN MARKET</t>
         </is>
       </c>
     </row>
     <row r="161" ht="20" customHeight="1">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>İNCESU MARKET</t>
+          <t>İKBAL TAVUK DÖNER -  KADİR YAVUZ</t>
         </is>
       </c>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>İNŞAAT MÜHENDİSLER ODASI ERZURUM ŞUBESİ.</t>
+          <t>İLYAS TOSUN</t>
         </is>
       </c>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>İRFAN GÜZELYURT  KÖŞEM DÜRÜM EVİ</t>
+          <t>İNCESU MARKET</t>
         </is>
       </c>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>İSHAK AYVAT - HACEGAN ŞÜKRÜPAŞA</t>
+          <t>İNŞAAT MÜHENDİSLER ODASI ERZURUM ŞUBESİ.</t>
         </is>
       </c>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>İS-MAR MARKET DURMUŞ TOKAT</t>
+          <t>İRFAN GÜZELYURT  KÖŞEM DÜRÜM EVİ</t>
         </is>
       </c>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>İSMODE MOBİLYA TARIM HAYV.İNŞ.TAAH.SAN.TİC.LTD.ŞTİ.</t>
+          <t>İSHAK AYVAT - HACEGAN ŞÜKRÜPAŞA</t>
         </is>
       </c>
     </row>
     <row r="167" ht="20" customHeight="1">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>İŞMAR - SALİH ZEKİ EMRAH İŞAŞIR</t>
+          <t>İS-MAR MARKET DURMUŞ TOKAT</t>
         </is>
       </c>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>KA ENERJİ ELEKTRİK TES.ENERJİ İNŞ.TAAH. NAK.GÜV.SİS.BİLİŞİM TEKN.SAN. VE LTD. ŞTİ.</t>
+          <t>İSMODE MOBİLYA TARIM HAYV.İNŞ.TAAH.SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>KAFKAS HOME ZÜCCACİYE VE PLASTİK SAN.TİC.LTD.ŞTİ.</t>
+          <t>İŞMAR - SALİH ZEKİ EMRAH İŞAŞIR</t>
         </is>
       </c>
     </row>
     <row r="170" ht="20" customHeight="1">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>KAHRAMANLAR ZÜCCACİYE</t>
+          <t>KA ENERJİ ELEKTRİK TES.ENERJİ İNŞ.TAAH. NAK.GÜV.SİS.BİLİŞİM TEKN.SAN. VE LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="171" ht="20" customHeight="1">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>KAR KİTAP KIRTASİYE - YASEMİN ÖZCOŞAR</t>
+          <t>KAFKAS HOME ZÜCCACİYE VE PLASTİK SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="172" ht="20" customHeight="1">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>KARACA GIDA - ERENTÜRK KARACA</t>
+          <t>KAHRAMANLAR ZÜCCACİYE</t>
         </is>
       </c>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>KARADENİZ BALIKCILIK</t>
+          <t>KAR KİTAP KIRTASİYE - YASEMİN ÖZCOŞAR</t>
         </is>
       </c>
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>KARALAR İNŞAAT LTD.ŞTİ.</t>
+          <t>KARACA GIDA - ERENTÜRK KARACA</t>
         </is>
       </c>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="2" t="inlineStr">
         <is>
+          <t>KARADENİZ BALIKCILIK</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="20" customHeight="1">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>KARALAR İNŞAAT LTD.ŞTİ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="20" customHeight="1">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
           <t>Karalar Toptan Gıda-
 Muammer Kara</t>
         </is>
       </c>
     </row>
-    <row r="176" ht="20" customHeight="1">
-      <c r="A176" s="2" t="inlineStr">
-        <is>
-          <t>KARBİR TEKSTİL İNŞAAT GIDA TEMİZLİK YEMEK NAKLİYE VE İTHALAT İHRACAT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="177" ht="20" customHeight="1">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>KARDELEN GRUP TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
-        </is>
-      </c>
-    </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>KARS CHOCOLADE</t>
+          <t>KARBİR TEKSTİL İNŞAAT GIDA TEMİZLİK YEMEK NAKLİYE VE İTHALAT İHRACAT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>KAYALAR KURUYEMİŞ</t>
+          <t>KARDELEN GRUP TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>KEBAPCI ÜSTADIM - MURAT EROL</t>
+          <t>KARS CHOCOLADE</t>
         </is>
       </c>
     </row>
     <row r="181" ht="20" customHeight="1">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>KELEŞOĞLU MARKET</t>
+          <t>KAYALAR KURUYEMİŞ</t>
         </is>
       </c>
     </row>
     <row r="182" ht="20" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>KERİM BEY HALISAHA</t>
+          <t>KEBAPCI ÜSTADIM - MURAT EROL</t>
         </is>
       </c>
     </row>
     <row r="183" ht="20" customHeight="1">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>KILIÇ MARKET - FATMA KILIÇ</t>
+          <t>KELEŞOĞLU MARKET</t>
         </is>
       </c>
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>KIRMIZI KÖŞEM</t>
+          <t>KERİM BEY HALISAHA</t>
         </is>
       </c>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>KİT-MAR KİTAP KIRTASİYE YAYIN DAĞITIM GIDA SANAYİ TİCARET ANONİM ŞİRKETİ</t>
+          <t>KILIÇ MARKET - FATMA KILIÇ</t>
         </is>
       </c>
     </row>
     <row r="186" ht="20" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>KOÇAKLAR MARKET - HALİT KOÇAK</t>
+          <t>KIRMIZI KÖŞEM</t>
         </is>
       </c>
     </row>
     <row r="187" ht="20" customHeight="1">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>KOÇHAN SÜT ÜRÜNLERİ SAN.TİC.LTD.ŞTİ.</t>
+          <t>KİT-MAR KİTAP KIRTASİYE YAYIN DAĞITIM GIDA SANAYİ TİCARET ANONİM ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="188" ht="20" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>KONAKLI ET RESTAORAN ZİGANA</t>
+          <t>KOÇAKLAR MARKET - HALİT KOÇAK</t>
         </is>
       </c>
     </row>
     <row r="189" ht="20" customHeight="1">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>KOTANOĞLU KİTAP KIRTASİYE TEMİZLİK MOBİLYA İNŞAAT TİCARET VE PAZARLAMA LİMİTED ŞİRKETİ</t>
+          <t>KOÇHAN SÜT ÜRÜNLERİ SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="190" ht="20" customHeight="1">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>KOTANOĞULLARI KİTAP KIRTASİYE  - VİLDAN KOTANOĞLU</t>
+          <t>KONAKLI ET RESTAORAN ZİGANA</t>
         </is>
       </c>
     </row>
     <row r="191" ht="20" customHeight="1">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>KÖŞEM MARKET - ENGİN AKAN</t>
+          <t>KOTANOĞLU KİTAP KIRTASİYE TEMİZLİK MOBİLYA İNŞAAT TİCARET VE PAZARLAMA LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="192" ht="20" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>KÖYCEĞİZ ŞARKÜTERİ - BETÜL RANA AYVAZ</t>
+          <t>KOTANOĞULLARI KİTAP KIRTASİYE  - VİLDAN KOTANOĞLU</t>
         </is>
       </c>
     </row>
     <row r="193" ht="20" customHeight="1">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>KREDİ BOÇLARI</t>
+          <t>KÖŞEM MARKET - ENGİN AKAN</t>
         </is>
       </c>
     </row>
     <row r="194" ht="20" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>KUDDUSİ BABA</t>
+          <t>KÖYCEĞİZ ŞARKÜTERİ - BETÜL RANA AYVAZ</t>
         </is>
       </c>
     </row>
     <row r="195" ht="20" customHeight="1">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>KURU AMBAR HÜSEYİN ABİ</t>
+          <t>KREDİ BOÇLARI</t>
         </is>
       </c>
     </row>
     <row r="196" ht="20" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>KUŞAK GIDA - SERVET KUŞUT</t>
+          <t>KUDDUSİ BABA</t>
         </is>
       </c>
     </row>
     <row r="197" ht="20" customHeight="1">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>KÜLTÜR A.Ş.</t>
+          <t>KURU AMBAR HÜSEYİN ABİ</t>
         </is>
       </c>
     </row>
     <row r="198" ht="20" customHeight="1">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>KÜLTÜR KIRTASİYE - AHMET TAŞCIOĞLU</t>
+          <t>KUŞAK GIDA - SERVET KUŞUT</t>
         </is>
       </c>
     </row>
     <row r="199" ht="20" customHeight="1">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>LAÇ KARDEŞLER TİC.SAN.LTD.ŞTİ.</t>
+          <t>KÜLTÜR A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="200" ht="20" customHeight="1">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>LAMPACARD LTD.ŞTİ.</t>
+          <t>KÜLTÜR KIRTASİYE - AHMET TAŞCIOĞLU</t>
         </is>
       </c>
     </row>
     <row r="201" ht="20" customHeight="1">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>LAPHARMA İLAÇ VETERİNERLİK İNŞAAT OTOMOTİV SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>LAÇ KARDEŞLER TİC.SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="202" ht="20" customHeight="1">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>LATİNOS MEKSİKA - ERTUĞTUL AKDOĞAN - TURAN AKSAKAL ADİ ORTAKLIK</t>
+          <t>LAMPACARD LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="203" ht="20" customHeight="1">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>LİDER MAĞAZACILIK TAŞ.PET.ÜRÜNLERİ MEDİKAL SAN.TİC.LTD.ŞTİ.</t>
+          <t>LAPHARMA İLAÇ VETERİNERLİK İNŞAAT OTOMOTİV SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="204" ht="20" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>LİMDAŞ HAVALANDIRMA TESİSAT İNŞAAT TAAHHÜT TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
+          <t>LATİNOS MEKSİKA - ERTUĞTUL AKDOĞAN - TURAN AKSAKAL ADİ ORTAKLIK</t>
         </is>
       </c>
     </row>
     <row r="205" ht="20" customHeight="1">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>MAHMUT UĞURLİ</t>
+          <t>LİDER MAĞAZACILIK TAŞ.PET.ÜRÜNLERİ MEDİKAL SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="206" ht="20" customHeight="1">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>MALAZGİRT KÖYLERE HİZMET GÖTÜRME BİRLİĞİ</t>
+          <t>LİMDAŞ HAVALANDIRMA TESİSAT İNŞAAT TAAHHÜT TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="207" ht="20" customHeight="1">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>MAREL TURİZM GIDA  LTD.ŞTİ.</t>
+          <t>MAHMUT UĞURLİ</t>
         </is>
       </c>
     </row>
     <row r="208" ht="20" customHeight="1">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>MATRAX SHOP</t>
+          <t>MALAZGİRT KÖYLERE HİZMET GÖTÜRME BİRLİĞİ</t>
         </is>
       </c>
     </row>
     <row r="209" ht="20" customHeight="1">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>MAVİ BİLİŞİM MUSTAFA BAKIRCI</t>
+          <t>MAREL TURİZM GIDA  LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="210" ht="20" customHeight="1">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>MAYA PASTANELERİ - ÖMER ATİK</t>
+          <t>MATRAX SHOP</t>
         </is>
       </c>
     </row>
     <row r="211" ht="20" customHeight="1">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>MEHMET BEY DOĞUBAYAZIT</t>
+          <t>MAVİ BİLİŞİM MUSTAFA BAKIRCI</t>
         </is>
       </c>
     </row>
     <row r="212" ht="20" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>MEHMET ÖZBAŞ</t>
+          <t>MAYA PASTANELERİ - ÖMER ATİK</t>
         </is>
       </c>
     </row>
     <row r="213" ht="20" customHeight="1">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>MEHMET SELİM KASIMOĞLU</t>
+          <t>MEHMET BEY DOĞUBAYAZIT</t>
         </is>
       </c>
     </row>
     <row r="214" ht="20" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>MEKKE PAZARI</t>
+          <t>MEHMET ÖZBAŞ</t>
         </is>
       </c>
     </row>
     <row r="215" ht="20" customHeight="1">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>MELİKE TEHTAP AYDIN - CHOCOLADE BOUTİQUE YILDIZKENT</t>
+          <t>MEHMET SELİM KASIMOĞLU</t>
         </is>
       </c>
     </row>
     <row r="216" ht="20" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>MEMİŞOĞULLARI TARIM İNŞAAT HAYVANCILIK NAKLİYE TİCARET İTHALAT İHRACAT LİMİTED ŞİRKET</t>
+          <t>MEKKE PAZARI</t>
         </is>
       </c>
     </row>
     <row r="217" ht="20" customHeight="1">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>MENA BİLİŞİM BİLGİSAYAR İLETİŞİM OTOMOTİV İNŞAAT TAAHHÜT TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
+          <t>MELİKE TEHTAP AYDIN - CHOCOLADE BOUTİQUE YILDIZKENT</t>
         </is>
       </c>
     </row>
     <row r="218" ht="20" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>MERAL KONFEKSİYON TİCARET LİMİTED ŞİRKETİ</t>
+          <t>MEMİŞOĞULLARI TARIM İNŞAAT HAYVANCILIK NAKLİYE TİCARET İTHALAT İHRACAT LİMİTED ŞİRKET</t>
         </is>
       </c>
     </row>
     <row r="219" ht="20" customHeight="1">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>MERVE YILDIZ GENCER</t>
+          <t>MENA BİLİŞİM BİLGİSAYAR İLETİŞİM OTOMOTİV İNŞAAT TAAHHÜT TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="220" ht="20" customHeight="1">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>MESA DAĞITIM PAZARLAMA - MERVE UNCUOĞLU</t>
+          <t>MERAL KONFEKSİYON TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="221" ht="20" customHeight="1">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>MESUT ÖZPEKER - HİRA ŞARKÜTERİ</t>
+          <t>MERVE YILDIZ GENCER</t>
         </is>
       </c>
     </row>
     <row r="222" ht="20" customHeight="1">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>METİN AKDAŞ - AKDAŞLAR MEYVE SEBZE BALIK</t>
+          <t>MESA DAĞITIM PAZARLAMA - MERVE UNCUOĞLU</t>
         </is>
       </c>
     </row>
     <row r="223" ht="20" customHeight="1">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>METİN GÜNEY - GÜNEYLER TOPTAN</t>
+          <t>MESUT ÖZPEKER - HİRA ŞARKÜTERİ</t>
         </is>
       </c>
     </row>
     <row r="224" ht="20" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>MİRAÇ KARTEPE ABDUSSAMED</t>
+          <t>METİN AKDAŞ - AKDAŞLAR MEYVE SEBZE BALIK</t>
         </is>
       </c>
     </row>
     <row r="225" ht="20" customHeight="1">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>MİRADAŞ TURİZM TAŞIMACILIK  ELEK.İNŞ.GIDA SAN.TİC.LTD. ŞTİ.</t>
+          <t>METİN GÜNEY - GÜNEYLER TOPTAN</t>
         </is>
       </c>
     </row>
     <row r="226" ht="20" customHeight="1">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>MİRKAY İNŞ.TAAH.VE SAN LTD.ŞTİ.</t>
+          <t>MİRAÇ KARTEPE ABDUSSAMED</t>
         </is>
       </c>
     </row>
     <row r="227" ht="20" customHeight="1">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>MMC EV TEKSTİL MOBİLYA ZÜCCACİYE İNŞ.TAAH.SANAYİ VE TİC.LTD.ŞTİ</t>
+          <t>MİRADAŞ TURİZM TAŞIMACILIK  ELEK.İNŞ.GIDA SAN.TİC.LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="228" ht="20" customHeight="1">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>MODA NİSA - ÇETİN ŞENOL</t>
+          <t>MİRKAY İNŞ.TAAH.VE SAN LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="229" ht="20" customHeight="1">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>MUAMMER USTA  -  MUAMMER TANHAŞ</t>
+          <t>MMC EV TEKSTİL MOBİLYA ZÜCCACİYE İNŞ.TAAH.SANAYİ VE TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="230" ht="20" customHeight="1">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>MUDİ GÜVENLİK</t>
+          <t>MODA NİSA - ÇETİN ŞENOL</t>
         </is>
       </c>
     </row>
     <row r="231" ht="20" customHeight="1">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>MUHAMMET EMİN YILMAZ - 3M ŞARKÜTERİ</t>
+          <t>MUAMMER USTA  -  MUAMMER TANHAŞ</t>
         </is>
       </c>
     </row>
     <row r="232" ht="20" customHeight="1">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>MUHAMMET SIDDIK ÇETRES-MEHMET AKİF ÇETRES-YUNUS EMRE ÇETRES ADİ ORTAKLIĞI</t>
+          <t>MUDİ GÜVENLİK</t>
         </is>
       </c>
     </row>
     <row r="233" ht="20" customHeight="1">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>MUHASEBE</t>
+          <t>MUHAMMET EMİN YILMAZ - 3M ŞARKÜTERİ</t>
         </is>
       </c>
     </row>
     <row r="234" ht="20" customHeight="1">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>MURAT POLAT</t>
+          <t>MUHAMMET SIDDIK ÇETRES-MEHMET AKİF ÇETRES-YUNUS EMRE ÇETRES ADİ ORTAKLIĞI</t>
         </is>
       </c>
     </row>
     <row r="235" ht="20" customHeight="1">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>murat usta</t>
+          <t>MUHASEBE</t>
         </is>
       </c>
     </row>
     <row r="236" ht="20" customHeight="1">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>MUSTAFA AKAL</t>
+          <t>MURAT POLAT</t>
         </is>
       </c>
     </row>
     <row r="237" ht="20" customHeight="1">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>MUSTAFA DEĞİRMENCİOĞLU</t>
+          <t>murat usta</t>
         </is>
       </c>
     </row>
     <row r="238" ht="20" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>MUSTAFA HALİL İBRAHİM GÜNALTIN - PEMBİŞ EV</t>
+          <t>MUSTAFA AKAL</t>
         </is>
       </c>
     </row>
     <row r="239" ht="20" customHeight="1">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>MUTLU AKÇAY</t>
+          <t>MUSTAFA DEĞİRMENCİOĞLU</t>
         </is>
       </c>
     </row>
     <row r="240" ht="20" customHeight="1">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>MÜR A.Ş.</t>
+          <t>MUSTAFA HALİL İBRAHİM GÜNALTIN - PEMBİŞ EV</t>
         </is>
       </c>
     </row>
     <row r="241" ht="20" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>MY SHOES RIFAT CAFE</t>
+          <t>MUTLU AKÇAY</t>
         </is>
       </c>
     </row>
     <row r="242" ht="20" customHeight="1">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>NAZAR KIRTASİYE</t>
+          <t>MÜR A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="243" ht="20" customHeight="1">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>NAZMİ MAZLUM GIDA PAZ.İNŞ.TAAH.NAKL.LTD.ŞTİ.</t>
+          <t>MY SHOES RIFAT CAFE</t>
         </is>
       </c>
     </row>
     <row r="244" ht="20" customHeight="1">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>NEFES KAFECİLİK - NEJLA TORUN</t>
+          <t>NAZAR KIRTASİYE</t>
         </is>
       </c>
     </row>
     <row r="245" ht="20" customHeight="1">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>NESA ÇOÇUK - NECLA  AKSU</t>
+          <t>NAZMİ MAZLUM GIDA PAZ.İNŞ.TAAH.NAKL.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="246" ht="20" customHeight="1">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>NEVA SAVUNMA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>NEFES KAFECİLİK - NEJLA TORUN</t>
         </is>
       </c>
     </row>
     <row r="247" ht="20" customHeight="1">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>NEW GROSS MARKETLER</t>
+          <t>NESA ÇOÇUK - NECLA  AKSU</t>
         </is>
       </c>
     </row>
     <row r="248" ht="20" customHeight="1">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Niasse Mobilya Ltd. Şti.</t>
+          <t>NEVA SAVUNMA SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="249" ht="20" customHeight="1">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>NİW GROSS MARKET- ALPARSLAN  BAYRAM</t>
+          <t>NEW GROSS MARKETLER</t>
         </is>
       </c>
     </row>
     <row r="250" ht="20" customHeight="1">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Nuh İnşaat Malz. İnş.Taah.Harf.Tic.San.Ltd.Şti.</t>
+          <t>Niasse Mobilya Ltd. Şti.</t>
         </is>
       </c>
     </row>
     <row r="251" ht="20" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>NUTRIALA GIDA SAN.VE TIC.LTD.STI.</t>
+          <t>NİW GROSS MARKET- ALPARSLAN  BAYRAM</t>
         </is>
       </c>
     </row>
     <row r="252" ht="20" customHeight="1">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>OKA GRUP GIDA İNŞAAT TURİZM TİCARET LTD.ŞTİ.</t>
+          <t>Nuh İnşaat Malz. İnş.Taah.Harf.Tic.San.Ltd.Şti.</t>
         </is>
       </c>
     </row>
     <row r="253" ht="20" customHeight="1">
       <c r="A253" s="2" t="inlineStr">
         <is>
-          <t>ONUR CAĞ KEBAP - NECMETTİN TOPŞAKLI</t>
+          <t>NUTRIALA GIDA SAN.VE TIC.LTD.STI.</t>
         </is>
       </c>
     </row>
     <row r="254" ht="20" customHeight="1">
       <c r="A254" s="2" t="inlineStr">
         <is>
-          <t>ORAL ET ENTEGRE A.Ş.</t>
+          <t>OKA GRUP GIDA İNŞAAT TURİZM TİCARET LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="255" ht="20" customHeight="1">
       <c r="A255" s="2" t="inlineStr">
         <is>
-          <t>ORHAN HOCA EYÜP</t>
+          <t>ONUR CAĞ KEBAP - NECMETTİN TOPŞAKLI</t>
         </is>
       </c>
     </row>
     <row r="256" ht="20" customHeight="1">
       <c r="A256" s="2" t="inlineStr">
         <is>
-          <t>OSMANAĞA LOKANTASI</t>
+          <t>ORAL ET ENTEGRE A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="257" ht="20" customHeight="1">
       <c r="A257" s="2" t="inlineStr">
         <is>
-          <t>OSMANLI GIDA İNŞ.TAAH.HAY.TEM.OTO.TİC. VE SAN.LTD.ŞTİ</t>
+          <t>ORHAN HOCA EYÜP</t>
         </is>
       </c>
     </row>
     <row r="258" ht="20" customHeight="1">
       <c r="A258" s="2" t="inlineStr">
         <is>
-          <t>ÖKKEŞ USTA</t>
+          <t>OSMANAĞA LOKANTASI</t>
         </is>
       </c>
     </row>
     <row r="259" ht="20" customHeight="1">
       <c r="A259" s="2" t="inlineStr">
         <is>
-          <t>ÖZ VATAN UNLU MAMULLER - SAMET ÇÜTELİ</t>
+          <t>OSMANLI GIDA İNŞ.TAAH.HAY.TEM.OTO.TİC. VE SAN.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="260" ht="20" customHeight="1">
       <c r="A260" s="2" t="inlineStr">
         <is>
-          <t>ÖZBEK PAZARLAMA</t>
+          <t>ÖKKEŞ USTA</t>
         </is>
       </c>
     </row>
     <row r="261" ht="20" customHeight="1">
       <c r="A261" s="2" t="inlineStr">
         <is>
-          <t>ÖZ-BEREKET MARKET - ÖMER FARUK TOHUMCU</t>
+          <t>ÖZ VATAN UNLU MAMULLER - SAMET ÇÜTELİ</t>
         </is>
       </c>
     </row>
     <row r="262" ht="20" customHeight="1">
       <c r="A262" s="2" t="inlineStr">
         <is>
-          <t>ÖZDEN BAL - MEHMET ÖZDEN</t>
+          <t>ÖZBEK PAZARLAMA</t>
         </is>
       </c>
     </row>
     <row r="263" ht="20" customHeight="1">
       <c r="A263" s="2" t="inlineStr">
         <is>
-          <t>PALANDÖKEN SAFİR TURİZM</t>
+          <t>ÖZ-BEREKET MARKET - ÖMER FARUK TOHUMCU</t>
         </is>
       </c>
     </row>
     <row r="264" ht="20" customHeight="1">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>PALANDÖKEN SAĞLIK HİZMETLERİ A.Ş.</t>
+          <t>ÖZDEN BAL - MEHMET ÖZDEN</t>
         </is>
       </c>
     </row>
     <row r="265" ht="20" customHeight="1">
       <c r="A265" s="2" t="inlineStr">
         <is>
-          <t>PALANDÖKEN SÜT</t>
+          <t>PALANDÖKEN SAFİR TURİZM</t>
         </is>
       </c>
     </row>
     <row r="266" ht="20" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>PATROON CAFE - BÜLENT AKYÜZ</t>
+          <t>PALANDÖKEN SAĞLIK HİZMETLERİ A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="267" ht="20" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>PERKON PERSONEL KONTROL BARKOD SİST. BİLG. YAZ. ELEKTRONİK TİC. SAN. A.Ş.</t>
+          <t>PALANDÖKEN SÜT</t>
         </is>
       </c>
     </row>
     <row r="268" ht="20" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>PERLA CAFE IĞDIR</t>
+          <t>PATROON CAFE - BÜLENT AKYÜZ</t>
         </is>
       </c>
     </row>
     <row r="269" ht="20" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>PEŞİN SATIŞLAR</t>
+          <t>PERKON PERSONEL KONTROL BARKOD SİST. BİLG. YAZ. ELEKTRONİK TİC. SAN. A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="270" ht="20" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>PEYNİR TATLISI ÖZCAN BEY</t>
+          <t>PERLA CAFE IĞDIR</t>
         </is>
       </c>
     </row>
     <row r="271" ht="20" customHeight="1">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>PİLAVCIM -MUHAMMED KOÇ</t>
+          <t>PEŞİN SATIŞLAR</t>
         </is>
       </c>
     </row>
     <row r="272" ht="20" customHeight="1">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>PİZZERİA - OKTAY TURNA</t>
+          <t>PEYNİR TATLISI ÖZCAN BEY</t>
         </is>
       </c>
     </row>
     <row r="273" ht="20" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>PİZZERİA -ERHAN ŞAHİN</t>
+          <t>PİLAVCIM -MUHAMMED KOÇ</t>
         </is>
       </c>
     </row>
     <row r="274" ht="20" customHeight="1">
       <c r="A274" s="2" t="inlineStr">
         <is>
-          <t>POLATLAR TİCARET - SALİH SARIPOLAT</t>
+          <t>PİZZERİA - OKTAY TURNA</t>
         </is>
       </c>
     </row>
     <row r="275" ht="20" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>POLATLAR YAZILIM LTD.ŞTİ.</t>
+          <t>PİZZERİA -ERHAN ŞAHİN</t>
         </is>
       </c>
     </row>
     <row r="276" ht="20" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>POLDİ TEKSTİL</t>
+          <t>POLATLAR TİCARET - SALİH SARIPOLAT</t>
         </is>
       </c>
     </row>
     <row r="277" ht="20" customHeight="1">
       <c r="A277" s="2" t="inlineStr">
         <is>
-          <t>POSSİFY BİLGİSAYAR VE OTOMASYON SİSTEMLERİ DIŞ. TİC. A.Ş.</t>
+          <t>POLATLAR YAZILIM LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="278" ht="20" customHeight="1">
       <c r="A278" s="2" t="inlineStr">
         <is>
-          <t>Propos Yazilim, Barkod ve Güvenlik Sistemleri</t>
+          <t>POLDİ TEKSTİL</t>
         </is>
       </c>
     </row>
     <row r="279" ht="20" customHeight="1">
       <c r="A279" s="2" t="inlineStr">
         <is>
-          <t>PROTEK BİLİŞİM BİLG.ELEKT.İNŞ.TAAH.MED.KIR.SAN.TİC.LTD.ŞTİ.</t>
+          <t>POSSİFY BİLGİSAYAR VE OTOMASYON SİSTEMLERİ DIŞ. TİC. A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="280" ht="20" customHeight="1">
       <c r="A280" s="2" t="inlineStr">
         <is>
-          <t>PURUT KIRTASİYE</t>
+          <t>Propos Yazilim, Barkod ve Güvenlik Sistemleri</t>
         </is>
       </c>
     </row>
     <row r="281" ht="20" customHeight="1">
       <c r="A281" s="2" t="inlineStr">
         <is>
-          <t>QR OBİRMENU</t>
+          <t>PROTEK BİLİŞİM BİLG.ELEKT.İNŞ.TAAH.MED.KIR.SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="282" ht="20" customHeight="1">
       <c r="A282" s="2" t="inlineStr">
         <is>
-          <t>RAMAZAN İLBEYLİ - TREND KIRTASİYE</t>
+          <t>PURUT KIRTASİYE</t>
         </is>
       </c>
     </row>
     <row r="283" ht="20" customHeight="1">
       <c r="A283" s="2" t="inlineStr">
         <is>
-          <t>REC GLOBAL ELEKTRONİK HIRDAVAT KOZMETİK OTOMOTİV SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>QR OBİRMENU</t>
         </is>
       </c>
     </row>
     <row r="284" ht="20" customHeight="1">
       <c r="A284" s="2" t="inlineStr">
         <is>
-          <t>RiPOSOFT-RIDVAN POLAT</t>
+          <t>RAMAZAN İLBEYLİ - TREND KIRTASİYE</t>
         </is>
       </c>
     </row>
     <row r="285" ht="20" customHeight="1">
       <c r="A285" s="2" t="inlineStr">
         <is>
-          <t>SADRA TURİZM GIDA SANAYİ TİCARET VE LİMİTED ŞİRKETİ</t>
+          <t>REC GLOBAL ELEKTRONİK HIRDAVAT KOZMETİK OTOMOTİV SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="286" ht="20" customHeight="1">
       <c r="A286" s="2" t="inlineStr">
         <is>
-          <t>SAĞLAM ECZANEZİ</t>
+          <t>RiPOSOFT-RIDVAN POLAT</t>
         </is>
       </c>
     </row>
     <row r="287" ht="20" customHeight="1">
       <c r="A287" s="2" t="inlineStr">
         <is>
-          <t>SALİH USTA PASTANESİ</t>
+          <t>SADRA TURİZM GIDA SANAYİ TİCARET VE LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="288" ht="20" customHeight="1">
       <c r="A288" s="2" t="inlineStr">
         <is>
-          <t>SALİM GIDA - MUSTAFA TOSUNOĞLU</t>
+          <t>SAĞLAM ECZANEZİ</t>
         </is>
       </c>
     </row>
     <row r="289" ht="20" customHeight="1">
       <c r="A289" s="2" t="inlineStr">
         <is>
-          <t>SANDAL MANAV VE BALIKÇILIK - LOKMAN AYDIN</t>
+          <t>SALİH USTA PASTANESİ</t>
         </is>
       </c>
     </row>
     <row r="290" ht="20" customHeight="1">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>SAYE BUTİK - ZEYNAP İME</t>
+          <t>SALİM GIDA - MUSTAFA TOSUNOĞLU</t>
         </is>
       </c>
     </row>
     <row r="291" ht="20" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>SB DİZAYN MAGAZİN MAĞAZALARI - BEDRİ SİNAN BUDAK</t>
+          <t>SANDAL MANAV VE BALIKÇILIK - LOKMAN AYDIN</t>
         </is>
       </c>
     </row>
     <row r="292" ht="20" customHeight="1">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>SECEDİT BİLGİSAYAR İLETİŞİM DANIŞMANLIK VE EĞİTİM HİZMETLERİ TİCARET LİMİTED ŞİRKETİ</t>
+          <t>SAYE BUTİK - ZEYNAP İME</t>
         </is>
       </c>
     </row>
     <row r="293" ht="20" customHeight="1">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>SEFA AKDAĞ</t>
+          <t>SB DİZAYN MAGAZİN MAĞAZALARI - BEDRİ SİNAN BUDAK</t>
         </is>
       </c>
     </row>
     <row r="294" ht="20" customHeight="1">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>SENA ÇAKAR - CEMRE KURUYEMİŞ</t>
+          <t>SECEDİT BİLGİSAYAR İLETİŞİM DANIŞMANLIK VE EĞİTİM HİZMETLERİ TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="295" ht="20" customHeight="1">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>SENSU TEMİZLİK ÜRÜN GIDA KOZMETİK PLASTİK NAK.TİC.SAN.LTD.ŞTİ.</t>
+          <t>SEFA AKDAĞ</t>
         </is>
       </c>
     </row>
     <row r="296" ht="20" customHeight="1">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>SERİNCE MAĞAZALARI LTD.ŞTİ.</t>
+          <t>SENA ÇAKAR - CEMRE KURUYEMİŞ</t>
         </is>
       </c>
     </row>
     <row r="297" ht="20" customHeight="1">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>SES AYDINLATMA ELEKTRİK İNŞ.TAAH.TEKS. PETROL SAN. TİC. LTD. ŞTİ.</t>
+          <t>SENSU TEMİZLİK ÜRÜN GIDA KOZMETİK PLASTİK NAK.TİC.SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="298" ht="20" customHeight="1">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>SES MAĞAZALARI GIDA ELEKTRİK VE ELEKTRONİK MALZEMELERİ TEKSTİL İNŞAAT TAAHHÜT TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
+          <t>SERİNCE MAĞAZALARI LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="299" ht="20" customHeight="1">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>SES TEKEL ÜRÜNLERİ DAĞITIM İLETİŞİM VE SAN. TİC.LTD.ŞTİ.</t>
+          <t>SES AYDINLATMA ELEKTRİK İNŞ.TAAH.TEKS. PETROL SAN. TİC. LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="300" ht="20" customHeight="1">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>SEVAL ŞEKERLEME GIDA SAN.TİC.LTD.ŞTİ</t>
+          <t>SES MAĞAZALARI GIDA ELEKTRİK VE ELEKTRONİK MALZEMELERİ TEKSTİL İNŞAAT TAAHHÜT TİCARET SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="301" ht="20" customHeight="1">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>SEVGİ KARAAL POLAT</t>
+          <t>SES TEKEL ÜRÜNLERİ DAĞITIM İLETİŞİM VE SAN. TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="302" ht="20" customHeight="1">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>SEVSER A.Ş.</t>
+          <t>SEVAL ŞEKERLEME GIDA SAN.TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="303" ht="20" customHeight="1">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>SEYHANLAR İNŞ.TURİZM.SEY.SAN.TİC.AŞ.</t>
+          <t>SEVGİ KARAAL POLAT</t>
         </is>
       </c>
     </row>
     <row r="304" ht="20" customHeight="1">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>SEZGIN GROSS TOPTAN PERAKENDE MARKETÇILIK INS.PETROL OTO TIC. LTD.STI.</t>
+          <t>SEVSER A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="305" ht="20" customHeight="1">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>SGK</t>
+          <t>SEYHANLAR İNŞ.TURİZM.SEY.SAN.TİC.AŞ.</t>
         </is>
       </c>
     </row>
     <row r="306" ht="20" customHeight="1">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>SIMIŞKA -İKRAM HOŞ</t>
+          <t>SEZGIN GROSS TOPTAN PERAKENDE MARKETÇILIK INS.PETROL OTO TIC. LTD.STI.</t>
         </is>
       </c>
     </row>
     <row r="307" ht="20" customHeight="1">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>SIRATAŞLAR KOZMETİK SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>SGK</t>
         </is>
       </c>
     </row>
     <row r="308" ht="20" customHeight="1">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>SİNAN GÜL - OSES</t>
+          <t>SIMIŞKA -İKRAM HOŞ</t>
         </is>
       </c>
     </row>
     <row r="309" ht="20" customHeight="1">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>SİSTEMLER.COM</t>
+          <t>SIRATAŞLAR KOZMETİK SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="310" ht="20" customHeight="1">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>SMZ TEMİZLİK GIDA İNŞAAT YEMEK İTHALAT İHRACAT SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
+          <t>SİNAN GÜL - OSES</t>
         </is>
       </c>
     </row>
     <row r="311" ht="20" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>SNR TAŞIMACILIK İNŞ.TAAH.PETROL TURİZM.OTOMOTİV.SAN.TİC.LTD.ŞTİ</t>
+          <t>SİSTEMLER.COM</t>
         </is>
       </c>
     </row>
     <row r="312" ht="20" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>Soner</t>
+          <t>SMZ TEMİZLİK GIDA İNŞAAT YEMEK İTHALAT İHRACAT SANAYİ VE TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="313" ht="20" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>SONER ISIYEL</t>
+          <t>SNR TAŞIMACILIK İNŞ.TAAH.PETROL TURİZM.OTOMOTİV.SAN.TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="314" ht="20" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>SONER YEDEKLEME SİSTEMİ</t>
+          <t>Soner</t>
         </is>
       </c>
     </row>
     <row r="315" ht="20" customHeight="1">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>SSK</t>
+          <t>SONER ISIYEL</t>
         </is>
       </c>
     </row>
     <row r="316" ht="20" customHeight="1">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>SUVARI</t>
+          <t>SONER YEDEKLEME SİSTEMİ</t>
         </is>
       </c>
     </row>
     <row r="317" ht="20" customHeight="1">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>ŞANCI MARKET - MÜNEVVER ŞANCI</t>
+          <t>SSK</t>
         </is>
       </c>
     </row>
     <row r="318" ht="20" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>ŞEMS ELEKTRİK</t>
+          <t>SUVARI</t>
         </is>
       </c>
     </row>
     <row r="319" ht="20" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>ŞENER GIDA</t>
+          <t>ŞANCI MARKET - MÜNEVVER ŞANCI</t>
         </is>
       </c>
     </row>
     <row r="320" ht="20" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>ŞENYURT CAĞ KEBAP- ALİ KARATAŞ</t>
+          <t>ŞEMS ELEKTRİK</t>
         </is>
       </c>
     </row>
     <row r="321" ht="20" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>TAB2 İNŞAAT GIDA OTOMOTİV HAYV.SAN.TİC.LTD.ŞTİ</t>
+          <t>ŞENER GIDA</t>
         </is>
       </c>
     </row>
     <row r="322" ht="20" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>TABYALAR GIDA HAYV. SAN.TIC.AS.</t>
+          <t>ŞENYURT CAĞ KEBAP- ALİ KARATAŞ</t>
         </is>
       </c>
     </row>
     <row r="323" ht="20" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>TAŞPINAR KURUYEMİŞ</t>
+          <t>TAB2 İNŞAAT GIDA OTOMOTİV HAYV.SAN.TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="324" ht="20" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>TATLI DİYARI- CABBAR AYDIN</t>
+          <t>TABYALAR GIDA HAYV. SAN.TIC.AS.</t>
         </is>
       </c>
     </row>
     <row r="325" ht="20" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>TAVŞANLI KURUYEMİŞ</t>
+          <t>TAŞPINAR KURUYEMİŞ</t>
         </is>
       </c>
     </row>
     <row r="326" ht="20" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>TEKLİF CARİSİ</t>
+          <t>TATLI DİYARI- CABBAR AYDIN</t>
         </is>
       </c>
     </row>
     <row r="327" ht="20" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>TEKNOKENT KOLEJİ</t>
+          <t>TAVŞANLI KURUYEMİŞ</t>
         </is>
       </c>
     </row>
     <row r="328" ht="20" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>TERMİNAL ÇORBACI</t>
+          <t>TEKLİF CARİSİ</t>
         </is>
       </c>
     </row>
     <row r="329" ht="20" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>TEZER YAPI İNŞAAT TAAHÜT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
+          <t>TEKNOKENT KOLEJİ</t>
         </is>
       </c>
     </row>
     <row r="330" ht="20" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>TMZ KAFE GIDA MEDIKAL İNŞ SAN.TİC.LTD.ŞTİ.</t>
+          <t>TERMİNAL ÇORBACI</t>
         </is>
       </c>
     </row>
     <row r="331" ht="20" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>TOPRAK MANAV</t>
+          <t>TEZER YAPI İNŞAAT TAAHÜT SANAYİ TİCARET LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="332" ht="20" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>TOST PEAK - TOLGA FEYZİOĞLU</t>
+          <t>TMZ KAFE GIDA MEDIKAL İNŞ SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="333" ht="20" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>TRABZON AS-AL BÖLGE BAŞKANLIĞI</t>
+          <t>TOPRAK MANAV</t>
         </is>
       </c>
     </row>
     <row r="334" ht="20" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>TRANSTUR PET.ÜR. İNŞ.TAH. REST.TEKS.GI.SAN.VE TİC.LTD.ŞTİ</t>
+          <t>TOST PEAK - TOLGA FEYZİOĞLU</t>
         </is>
       </c>
     </row>
     <row r="335" ht="20" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>TREND KIRTASİYE</t>
+          <t>TRABZON AS-AL BÖLGE BAŞKANLIĞI</t>
         </is>
       </c>
     </row>
     <row r="336" ht="20" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>TURAN TEKNOLOJİ</t>
+          <t>TRANSTUR PET.ÜR. İNŞ.TAH. REST.TEKS.GI.SAN.VE TİC.LTD.ŞTİ</t>
         </is>
       </c>
     </row>
     <row r="337" ht="20" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>TURHAN DİNLER</t>
+          <t>TREND KIRTASİYE</t>
         </is>
       </c>
     </row>
     <row r="338" ht="20" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>TURHAN DİNLER-CİVCİX CHİCKEN</t>
+          <t>TURAN TEKNOLOJİ</t>
         </is>
       </c>
     </row>
     <row r="339" ht="20" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>Turkcell İletişim Hizmetleri A.Ş.</t>
+          <t>TURHAN DİNLER</t>
         </is>
       </c>
     </row>
     <row r="340" ht="20" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>TURKISH HOME - EMRAH YILDIRIM</t>
+          <t>TURHAN DİNLER-CİVCİX CHİCKEN</t>
         </is>
       </c>
     </row>
     <row r="341" ht="20" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>UFUK ELEKTRİK - UFUK ŞİŞECİ</t>
+          <t>Turkcell İletişim Hizmetleri A.Ş.</t>
         </is>
       </c>
     </row>
     <row r="342" ht="20" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>UĞUR TARHAN</t>
+          <t>TURKISH HOME - EMRAH YILDIRIM</t>
         </is>
       </c>
     </row>
     <row r="343" ht="20" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>UNİKON GÜVENLİK TEKNOLOJİLERİ SAN.TİC.LTD.ŞTİ.</t>
+          <t>UFUK ELEKTRİK - UFUK ŞİŞECİ</t>
         </is>
       </c>
     </row>
     <row r="344" ht="20" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>UNİNET TELEKOM LTD.ŞTİ.</t>
+          <t>UĞUR TARHAN</t>
         </is>
       </c>
     </row>
     <row r="345" ht="20" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>ÜÇ YILDIZ HIRDAVAT İTH.İHR. SAN. TİC. LTD. ŞTİ.</t>
+          <t>UNİKON GÜVENLİK TEKNOLOJİLERİ SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="346" ht="20" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>ÜNİNET TELEKOM BİLGİSAYAR TELEKOMÜNİKASYON</t>
+          <t>UNİNET TELEKOM LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="347" ht="20" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>VAN SÜT</t>
+          <t>ÜÇ YILDIZ HIRDAVAT İTH.İHR. SAN. TİC. LTD. ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="348" ht="20" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>VEFA DİŞ DEPOSU İNŞ.SAN.TİC.LTD.ŞTİ.</t>
+          <t>ÜNİNET TELEKOM BİLGİSAYAR TELEKOMÜNİKASYON</t>
         </is>
       </c>
     </row>
     <row r="349" ht="20" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>VERGİ DAİRESİ POLATLAR</t>
+          <t>VAN SÜT</t>
         </is>
       </c>
     </row>
     <row r="350" ht="20" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>VIRAAGLASS CAM TICARET SANAYI LTD.STI.</t>
+          <t>VEFA DİŞ DEPOSU İNŞ.SAN.TİC.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="351" ht="20" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>VİOLET PLUS - BARIŞ YILMAZ</t>
+          <t>VERGİ DAİRESİ POLATLAR</t>
         </is>
       </c>
     </row>
     <row r="352" ht="20" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>VİOLET XL - ÇİĞDEM ESRA ŞAHİN</t>
+          <t>VIRAAGLASS CAM TICARET SANAYI LTD.STI.</t>
         </is>
       </c>
     </row>
     <row r="353" ht="20" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>YAHYA AYVAT</t>
+          <t>VİOLET PLUS - BARIŞ YILMAZ</t>
         </is>
       </c>
     </row>
     <row r="354" ht="20" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>YANKILAR MÜHENDİSLİK İNŞAAT TAAHHÜT ELEKTRİK DOĞALGAZ TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
+          <t>VİOLET XL - ÇİĞDEM ESRA ŞAHİN</t>
         </is>
       </c>
     </row>
     <row r="355" ht="20" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>YAPICI KROM SAN.LTD.ŞTİ.</t>
+          <t>YAHYA AYVAT</t>
         </is>
       </c>
     </row>
     <row r="356" ht="20" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>YAŞAM MARKET LTD.ŞTİ.</t>
+          <t>YANKILAR MÜHENDİSLİK İNŞAAT TAAHHÜT ELEKTRİK DOĞALGAZ TİCARET VE SANAYİ LİMİTED ŞİRKETİ</t>
         </is>
       </c>
     </row>
     <row r="357" ht="20" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>YEŞİL VİTAMİN MANAVI</t>
+          <t>YAPAY ZEKA BURAK</t>
         </is>
       </c>
     </row>
     <row r="358" ht="20" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>YILDIZ MARKET - HORASAN</t>
+          <t>YAPICI KROM SAN.LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="359" ht="20" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>YILDIZHAN TİCARET SÜT ÜRÜNLERİ LTD.ŞTİ.</t>
+          <t>YAŞAM MARKET LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="360" ht="20" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>YILMAR DEMİROZU</t>
+          <t>YEŞİL VİTAMİN MANAVI</t>
         </is>
       </c>
     </row>
     <row r="361" ht="20" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>YİĞİT MARKET İSPİR</t>
+          <t>YILDIZ MARKET - HORASAN</t>
         </is>
       </c>
     </row>
     <row r="362" ht="20" customHeight="1">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>YİĞİT-ER EKMEKÇİLİK GIDA NAKLİYE SANAYİ VE TİCARET LTD.ŞTİ.</t>
+          <t>YILDIZHAN TİCARET SÜT ÜRÜNLERİ LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="363" ht="20" customHeight="1">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>YUMAK TUHAFİYE</t>
+          <t>YILMAR DEMİROZU</t>
         </is>
       </c>
     </row>
     <row r="364" ht="20" customHeight="1">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>YUNUS EMRE AYVAT -HACEGAN MISIR ÇARŞISI</t>
+          <t>YİĞİT MARKET İSPİR</t>
         </is>
       </c>
     </row>
     <row r="365" ht="20" customHeight="1">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>Yurtiçi Kargo Servisi A.Ş. Genel Müdürlük</t>
+          <t>YİĞİT-ER EKMEKÇİLİK GIDA NAKLİYE SANAYİ VE TİCARET LTD.ŞTİ.</t>
         </is>
       </c>
     </row>
     <row r="366" ht="20" customHeight="1">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>YUSUF-EMRE ÇİZMELİOĞLU ORT</t>
+          <t>YUMAK TUHAFİYE</t>
         </is>
       </c>
     </row>
     <row r="367" ht="20" customHeight="1">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>ZAFER ABİ</t>
+          <t>YUNUS EMRE AYVAT -HACEGAN MISIR ÇARŞISI</t>
         </is>
       </c>
     </row>
     <row r="368" ht="20" customHeight="1">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>ZAFER DEMİR</t>
+          <t>Yurtiçi Kargo Servisi A.Ş. Genel Müdürlük</t>
         </is>
       </c>
     </row>
     <row r="369" ht="20" customHeight="1">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>ZARAFET KONFEKSİYON - SERHAT DEĞİRMENCİOĞLU</t>
+          <t>YUSUF-EMRE ÇİZMELİOĞLU ORT</t>
         </is>
       </c>
     </row>
     <row r="370" ht="20" customHeight="1">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>ZEYNEP SUSEVEN</t>
+          <t>ZAFER ABİ</t>
         </is>
       </c>
     </row>
     <row r="371" ht="20" customHeight="1">
       <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>ZAFER DEMİR</t>
+        </is>
+      </c>
+    </row>
+    <row r="372" ht="20" customHeight="1">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>ZARAFET KONFEKSİYON - SERHAT DEĞİRMENCİOĞLU</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" ht="20" customHeight="1">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>ZEYNEP SUSEVEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="20" customHeight="1">
+      <c r="A374" s="2" t="inlineStr">
         <is>
           <t>ZULEYHA KARAAL</t>
         </is>

</xml_diff>